<commit_message>
Improve DRM PPTX export and local upload launcher
</commit_message>
<xml_diff>
--- a/exports/Moradabad_Division_DRM_Budget_FR_Analysis.xlsx
+++ b/exports/Moradabad_Division_DRM_Budget_FR_Analysis.xlsx
@@ -487,9 +487,9 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -631,7 +631,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>109 🔴</t>
+          <t>109</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>36 🟢</t>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>122 🔴</t>
+          <t>122</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>41 🟢</t>
+          <t>41</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>126 🔴</t>
+          <t>126</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t>42 🟢</t>
+          <t>42</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>160 🔴</t>
+          <t>160</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -798,7 +798,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>53 🟢</t>
+          <t>53</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>117 🔴</t>
+          <t>117</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>39 🟢</t>
+          <t>39</t>
         </is>
       </c>
     </row>
@@ -891,7 +891,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>140 🔴</t>
+          <t>140</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>47 🟢</t>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>120 🔴</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>40 🟢</t>
+          <t>40</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>92 🟠</t>
+          <t>92</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>31 🟢</t>
+          <t>31</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>174 🔴</t>
+          <t>174</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>58 🟢</t>
+          <t>58</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>107 🔴</t>
+          <t>107</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>36 🟢</t>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>99 🟠</t>
+          <t>99</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>33 🟢</t>
+          <t>33</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>115 🔴</t>
+          <t>115</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>38 🟢</t>
+          <t>38</t>
         </is>
       </c>
     </row>
@@ -1251,7 +1251,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>-36084 🟢</t>
+          <t>-36084</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>-12028 🟢</t>
+          <t>-12028</t>
         </is>
       </c>
     </row>
@@ -1417,7 +1417,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>110 🔴</t>
+          <t>110</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1428,7 +1428,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>37 🟢</t>
+          <t>37</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1464,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>116 🔴</t>
+          <t>116</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>39 🟢</t>
+          <t>39</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>0 🟢</t>
+          <t>0</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1522,7 +1522,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>0 🟢</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>104 🔴</t>
+          <t>104</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>35 🟢</t>
+          <t>35</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>105 🔴</t>
+          <t>105</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>35 🟢</t>
+          <t>35</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>128 🔴</t>
+          <t>128</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>43 🟢</t>
+          <t>43</t>
         </is>
       </c>
     </row>
@@ -1699,7 +1699,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>212 🔴</t>
+          <t>212</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>71 🟢</t>
+          <t>71</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>140 🔴</t>
+          <t>140</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>47 🟢</t>
+          <t>47</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>143 🔴</t>
+          <t>143</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>48 🟢</t>
+          <t>48</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>172 🔴</t>
+          <t>172</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>57 🟢</t>
+          <t>57</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>172 🔴</t>
+          <t>172</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>57 🟢</t>
+          <t>57</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>283 🔴</t>
+          <t>283</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>94 🟠</t>
+          <t>94</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>118 🔴</t>
+          <t>118</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>39 🟢</t>
+          <t>39</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>165 🔴</t>
+          <t>165</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>55 🟢</t>
+          <t>55</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>126 🔴</t>
+          <t>126</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>42 🟢</t>
+          <t>42</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>85 🟠</t>
+          <t>85</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>28 🟢</t>
+          <t>28</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>153 🔴</t>
+          <t>153</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>51 🟢</t>
+          <t>51</t>
         </is>
       </c>
     </row>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>115 🔴</t>
+          <t>115</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -2346,7 +2346,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>38 🟢</t>
+          <t>38</t>
         </is>
       </c>
     </row>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>120 🔴</t>
+          <t>120</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>40 🟢</t>
+          <t>40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align exports with portal BP calculations
</commit_message>
<xml_diff>
--- a/exports/Moradabad_Division_DRM_Budget_FR_Analysis.xlsx
+++ b/exports/Moradabad_Division_DRM_Budget_FR_Analysis.xlsx
@@ -613,8 +613,8 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>213,841
-Cr. 21.38</t>
+          <t>240,031
+Cr. 24.00</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -625,13 +625,13 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>18,753
-Cr. 1.88</t>
+          <t>-7,437
+Cr. -0.74</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>97</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -665,8 +665,8 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>1,202,967
-Cr. 120.30</t>
+          <t>1,177,984
+Cr. 117.80</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -677,13 +677,13 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>264,851
-Cr. 26.49</t>
+          <t>289,834
+Cr. 28.98</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>122</t>
+          <t>125</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -717,8 +717,8 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>621,614
-Cr. 62.16</t>
+          <t>923,741
+Cr. 92.37</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -729,13 +729,13 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>160,418
-Cr. 16.04</t>
+          <t>-141,709
+Cr. -14.17</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>85</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -769,8 +769,8 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>451,194
-Cr. 45.12</t>
+          <t>413,960
+Cr. 41.40</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -781,13 +781,13 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>271,412
-Cr. 27.14</t>
+          <t>308,646
+Cr. 30.86</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>175</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -821,8 +821,8 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>686,650
-Cr. 68.67</t>
+          <t>694,140
+Cr. 69.41</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -833,13 +833,13 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>113,462
-Cr. 11.35</t>
+          <t>105,972
+Cr. 10.60</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>117</t>
+          <t>115</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -873,8 +873,8 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>1,117,522
-Cr. 111.75</t>
+          <t>1,217,272
+Cr. 121.73</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -885,13 +885,13 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>445,441
-Cr. 44.54</t>
+          <t>345,691
+Cr. 34.57</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>128</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -925,8 +925,8 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1,476,255
-Cr. 147.63</t>
+          <t>1,511,191
+Cr. 151.12</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -937,13 +937,13 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>301,046
-Cr. 30.10</t>
+          <t>266,110
+Cr. 26.61</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>118</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -977,8 +977,8 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>3,869,069
-Cr. 386.91</t>
+          <t>3,862,305
+Cr. 386.23</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -989,8 +989,8 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>-323,855
-Cr. -32.39</t>
+          <t>-317,091
+Cr. -31.71</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1029,8 +1029,8 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>464,277
-Cr. 46.43</t>
+          <t>598,674
+Cr. 59.87</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1041,13 +1041,13 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>343,473
-Cr. 34.35</t>
+          <t>209,076
+Cr. 20.91</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>135</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1081,8 +1081,8 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>331,546
-Cr. 33.15</t>
+          <t>325,688
+Cr. 32.57</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1093,13 +1093,13 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>24,320
-Cr. 2.43</t>
+          <t>30,178
+Cr. 3.02</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>109</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
@@ -1133,8 +1133,8 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>430,356
-Cr. 43.04</t>
+          <t>388,570
+Cr. 38.86</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1145,13 +1145,13 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>-4,678
-Cr. -0.47</t>
+          <t>37,108
+Cr. 3.71</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>110</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
@@ -1181,8 +1181,8 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>10,865,291
-Cr. 1086.53</t>
+          <t>11,353,556
+Cr. 1135.36</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1193,13 +1193,13 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>1,614,643
-Cr. 161.46</t>
+          <t>1,126,378
+Cr. 112.64</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>110</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
@@ -1233,8 +1233,8 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>-4,348
-Cr. -0.43</t>
+          <t>1,362,799
+Cr. 136.28</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1245,13 +1245,13 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>1,573,380
-Cr. 157.34</t>
+          <t>206,233
+Cr. 20.62</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>-36084</t>
+          <t>115</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1399,8 +1399,8 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2,235,470
-Cr. 223.55</t>
+          <t>2,249,064
+Cr. 224.91</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -1411,13 +1411,13 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>219,422
-Cr. 21.94</t>
+          <t>205,828
+Cr. 20.58</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>109</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1446,8 +1446,8 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>1,366,818
-Cr. 136.68</t>
+          <t>1,359,404
+Cr. 135.94</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1458,8 +1458,8 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>213,027
-Cr. 21.30</t>
+          <t>220,441
+Cr. 22.04</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
@@ -1493,8 +1493,8 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>95,030
-Cr. 9.50</t>
+          <t>0
+Cr. 0.00</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1505,8 +1505,8 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>-94,949
-Cr. -9.49</t>
+          <t>81
+Cr. 0.01</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1540,8 +1540,8 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>258,733
-Cr. 25.87</t>
+          <t>268,852
+Cr. 26.89</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1552,13 +1552,13 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>11,258
-Cr. 1.13</t>
+          <t>1,139
+Cr. 0.11</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>100</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1587,8 +1587,8 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>165,536
-Cr. 16.55</t>
+          <t>167,312
+Cr. 16.73</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1599,13 +1599,13 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>7,971
-Cr. 0.80</t>
+          <t>6,195
+Cr. 0.62</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>105</t>
+          <t>104</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1634,8 +1634,8 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>226,732
-Cr. 22.67</t>
+          <t>255,207
+Cr. 25.52</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1646,13 +1646,13 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>63,750
-Cr. 6.37</t>
+          <t>35,275
+Cr. 3.53</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>114</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1681,8 +1681,8 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>25,767
-Cr. 2.58</t>
+          <t>26,924
+Cr. 2.69</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -1693,13 +1693,13 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>28,778
-Cr. 2.88</t>
+          <t>27,621
+Cr. 2.76</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>203</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -1728,8 +1728,8 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>69,971
-Cr. 7.00</t>
+          <t>69,543
+Cr. 6.95</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1740,13 +1740,13 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>28,051
-Cr. 2.81</t>
+          <t>28,479
+Cr. 2.85</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>140</t>
+          <t>141</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1775,8 +1775,8 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>175,944
-Cr. 17.59</t>
+          <t>273,477
+Cr. 27.35</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1787,13 +1787,13 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>74,849
-Cr. 7.48</t>
+          <t>-22,684
+Cr. -2.27</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>143</t>
+          <t>92</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1822,8 +1822,8 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>5,349
-Cr. 0.53</t>
+          <t>5,665
+Cr. 0.57</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1834,13 +1834,13 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>3,828
-Cr. 0.38</t>
+          <t>3,512
+Cr. 0.35</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>162</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1869,8 +1869,8 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>102,694
-Cr. 10.27</t>
+          <t>100,083
+Cr. 10.01</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -1881,13 +1881,13 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>73,426
-Cr. 7.34</t>
+          <t>76,037
+Cr. 7.60</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>172</t>
+          <t>176</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -1916,8 +1916,8 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>126,473
-Cr. 12.65</t>
+          <t>320,448
+Cr. 32.04</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -1928,13 +1928,13 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>231,982
-Cr. 23.20</t>
+          <t>38,007
+Cr. 3.80</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>283</t>
+          <t>112</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -1963,8 +1963,8 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>4,854,516
-Cr. 485.45</t>
+          <t>5,095,979
+Cr. 509.60</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -1975,13 +1975,13 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>861,394
-Cr. 86.14</t>
+          <t>619,931
+Cr. 61.99</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>112</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -2129,8 +2129,8 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>356,251
-Cr. 35.63</t>
+          <t>350,722
+Cr. 35.07</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -2141,13 +2141,13 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>232,066
-Cr. 23.21</t>
+          <t>237,595
+Cr. 23.76</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>165</t>
+          <t>168</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -2176,8 +2176,8 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>49,982
-Cr. 5.00</t>
+          <t>52,719
+Cr. 5.27</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -2188,13 +2188,13 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>13,037
-Cr. 1.30</t>
+          <t>10,300
+Cr. 1.03</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>120</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -2223,8 +2223,8 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1,292,908
-Cr. 129.29</t>
+          <t>1,330,274
+Cr. 133.03</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -2235,13 +2235,13 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>-192,688
-Cr. -19.27</t>
+          <t>-230,054
+Cr. -23.01</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>83</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -2270,8 +2270,8 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>1,084,770
-Cr. 108.48</t>
+          <t>1,396,328
+Cr. 139.63</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -2282,13 +2282,13 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>573,697
-Cr. 57.37</t>
+          <t>262,139
+Cr. 26.21</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>153</t>
+          <t>119</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -2317,8 +2317,8 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>1,567,785
-Cr. 156.78</t>
+          <t>1,538,432
+Cr. 153.84</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -2329,13 +2329,13 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>239,289
-Cr. 23.93</t>
+          <t>268,642
+Cr. 26.86</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>115</t>
+          <t>117</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -2364,8 +2364,8 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>4,351,696
-Cr. 435.17</t>
+          <t>4,668,475
+Cr. 466.85</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -2376,13 +2376,13 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>865,401
-Cr. 86.54</t>
+          <t>548,622
+Cr. 54.86</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>112</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">

</xml_diff>